<commit_message>
chore(valuation): 밸류에이션 스냅샷 2026-08-15
</commit_message>
<xml_diff>
--- a/telegram_research_dashboard/static/valuation_full.xlsx
+++ b/telegram_research_dashboard/static/valuation_full.xlsx
@@ -4568,56 +4568,56 @@
         <v>4465</v>
       </c>
       <c r="C54" s="9" t="n">
-        <v>0</v>
+        <v>5.38</v>
       </c>
       <c r="D54" s="9" t="n">
-        <v>0</v>
+        <v>5.48</v>
       </c>
       <c r="E54" s="9" t="n">
-        <v>0.01</v>
+        <v>7.35</v>
       </c>
       <c r="F54" s="9" t="n">
-        <v>0.01</v>
+        <v>13.73</v>
       </c>
       <c r="G54" s="10" t="n">
-        <v>0.01</v>
+        <v>10.7</v>
       </c>
       <c r="H54" s="10" t="n">
-        <v>0.01</v>
+        <v>9.98</v>
       </c>
       <c r="I54" s="10" t="n"/>
       <c r="J54" s="9" t="n">
-        <v>0.68</v>
+        <v>3.59</v>
       </c>
       <c r="K54" s="9" t="n">
-        <v>0.01</v>
+        <v>3.14</v>
       </c>
       <c r="L54" s="9" t="n">
-        <v>0.16</v>
+        <v>3.61</v>
       </c>
       <c r="M54" s="9" t="n">
-        <v>-0.28</v>
+        <v>5.3</v>
       </c>
       <c r="N54" s="10" t="n"/>
       <c r="O54" s="10" t="n"/>
       <c r="P54" s="10" t="n"/>
       <c r="Q54" s="9" t="n">
-        <v>0</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="R54" s="9" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="S54" s="9" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="T54" s="9" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="U54" s="10" t="n">
-        <v>0</v>
+        <v>0.84</v>
       </c>
       <c r="V54" s="10" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="W54" s="10" t="n"/>
       <c r="X54" s="11" t="n">
@@ -4640,22 +4640,22 @@
       </c>
       <c r="AD54" s="12" t="n"/>
       <c r="AE54" s="9" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="AF54" s="9" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="AG54" s="9" t="n">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="AH54" s="9" t="n">
-        <v>0</v>
+        <v>0.63</v>
       </c>
       <c r="AI54" s="10" t="n">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="AJ54" s="10" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="AK54" s="10" t="n"/>
     </row>
@@ -5753,7 +5753,7 @@
         </is>
       </c>
       <c r="B70" s="8" t="n">
-        <v>172406</v>
+        <v>25569</v>
       </c>
       <c r="C70" s="9" t="n">
         <v>31.28</v>
@@ -5854,7 +5854,7 @@
         </is>
       </c>
       <c r="B71" s="8" t="n">
-        <v>93906</v>
+        <v>13927</v>
       </c>
       <c r="C71" s="9" t="n">
         <v>13.89</v>
@@ -5959,32 +5959,32 @@
         <v>6.51</v>
       </c>
       <c r="D72" s="15" t="n">
-        <v>6</v>
+        <v>6.27</v>
       </c>
       <c r="E72" s="15" t="n">
-        <v>5.58</v>
+        <v>7.35</v>
       </c>
       <c r="F72" s="15" t="n">
-        <v>5.89</v>
+        <v>8.390000000000001</v>
       </c>
       <c r="G72" s="15" t="n">
-        <v>8.390000000000001</v>
+        <v>10.29</v>
       </c>
       <c r="H72" s="15" t="n">
-        <v>6.89</v>
+        <v>9.34</v>
       </c>
       <c r="I72" s="15" t="n"/>
       <c r="J72" s="15" t="n">
-        <v>3.48</v>
+        <v>3.77</v>
       </c>
       <c r="K72" s="15" t="n">
-        <v>3.03</v>
+        <v>3.35</v>
       </c>
       <c r="L72" s="15" t="n">
-        <v>2.65</v>
+        <v>3.56</v>
       </c>
       <c r="M72" s="15" t="n">
-        <v>3.77</v>
+        <v>5.07</v>
       </c>
       <c r="N72" s="15" t="n"/>
       <c r="O72" s="15" t="n"/>
@@ -5993,13 +5993,13 @@
         <v>0.8100000000000001</v>
       </c>
       <c r="R72" s="15" t="n">
-        <v>0.6</v>
+        <v>0.73</v>
       </c>
       <c r="S72" s="15" t="n">
-        <v>0.46</v>
+        <v>0.55</v>
       </c>
       <c r="T72" s="15" t="n">
-        <v>0.52</v>
+        <v>0.66</v>
       </c>
       <c r="U72" s="15" t="n">
         <v>0.9</v>
@@ -6028,22 +6028,22 @@
       </c>
       <c r="AD72" s="16" t="n"/>
       <c r="AE72" s="15" t="n">
-        <v>0.33</v>
+        <v>0.37</v>
       </c>
       <c r="AF72" s="15" t="n">
-        <v>0.3</v>
+        <v>0.37</v>
       </c>
       <c r="AG72" s="15" t="n">
-        <v>0.31</v>
+        <v>0.35</v>
       </c>
       <c r="AH72" s="15" t="n">
-        <v>0.43</v>
+        <v>0.53</v>
       </c>
       <c r="AI72" s="15" t="n">
-        <v>0.57</v>
+        <v>0.66</v>
       </c>
       <c r="AJ72" s="15" t="n">
-        <v>0.51</v>
+        <v>0.64</v>
       </c>
       <c r="AK72" s="15" t="n"/>
     </row>
@@ -7823,22 +7823,22 @@
         <v>4465</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>0</v>
+        <v>5.38</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>0</v>
+        <v>5.48</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.01</v>
+        <v>7.35</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>0.01</v>
+        <v>13.73</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>0.01</v>
+        <v>10.7</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>0.01</v>
+        <v>9.98</v>
       </c>
       <c r="L29" s="9" t="n"/>
     </row>
@@ -8164,7 +8164,7 @@
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>172406</v>
+        <v>25569</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>31.28</v>
@@ -8208,7 +8208,7 @@
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>93906</v>
+        <v>13927</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>13.89</v>
@@ -9573,16 +9573,16 @@
         <v>4465</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>0.68</v>
+        <v>3.59</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>0.01</v>
+        <v>3.14</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0.16</v>
+        <v>3.61</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>-0.28</v>
+        <v>5.3</v>
       </c>
       <c r="J29" s="9" t="n"/>
       <c r="K29" s="9" t="n"/>
@@ -9890,7 +9890,7 @@
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>172406</v>
+        <v>25569</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>18.39</v>
@@ -9930,7 +9930,7 @@
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>93906</v>
+        <v>13927</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>7.78</v>
@@ -11397,22 +11397,22 @@
         <v>4465</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>0</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>0</v>
+        <v>0.84</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="L29" s="9" t="n"/>
     </row>
@@ -11742,7 +11742,7 @@
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>172406</v>
+        <v>25569</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>2.06</v>
@@ -11786,7 +11786,7 @@
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>93906</v>
+        <v>13927</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>1.12</v>
@@ -13620,7 +13620,7 @@
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>172406</v>
+        <v>25569</v>
       </c>
       <c r="F37" s="11" t="n">
         <v>6.6</v>
@@ -13664,7 +13664,7 @@
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>93906</v>
+        <v>13927</v>
       </c>
       <c r="F38" s="11" t="n">
         <v>8.1</v>
@@ -15143,22 +15143,22 @@
         <v>4465</v>
       </c>
       <c r="F29" s="9" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="I29" s="9" t="n">
-        <v>0</v>
+        <v>0.63</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="L29" s="9" t="n"/>
     </row>
@@ -15488,7 +15488,7 @@
         </is>
       </c>
       <c r="E37" s="7" t="n">
-        <v>172406</v>
+        <v>25569</v>
       </c>
       <c r="F37" s="9" t="n">
         <v>1.66</v>
@@ -15532,7 +15532,7 @@
         </is>
       </c>
       <c r="E38" s="7" t="n">
-        <v>93906</v>
+        <v>13927</v>
       </c>
       <c r="F38" s="9" t="n">
         <v>0.64</v>
@@ -24633,7 +24633,7 @@
         <v>60.72</v>
       </c>
       <c r="J126" s="18" t="n">
-        <v>85308163680</v>
+        <v>85308175580</v>
       </c>
       <c r="K126" s="18" t="n">
         <v>7485538259.999999</v>
@@ -29259,19 +29259,19 @@
         <v>5024387667000</v>
       </c>
       <c r="M191" s="7" t="n">
-        <v>0</v>
+        <v>5.38</v>
       </c>
       <c r="N191" s="7" t="n">
-        <v>0.68</v>
+        <v>3.59</v>
       </c>
       <c r="O191" s="7" t="n">
-        <v>0</v>
+        <v>0.6899999999999999</v>
       </c>
       <c r="P191" s="7" t="n">
         <v>12.82</v>
       </c>
       <c r="Q191" s="7" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="R191" s="7" t="inlineStr">
         <is>
@@ -29334,19 +29334,19 @@
         <v>5954812811000</v>
       </c>
       <c r="M192" s="7" t="n">
-        <v>0</v>
+        <v>5.48</v>
       </c>
       <c r="N192" s="7" t="n">
-        <v>0.01</v>
+        <v>3.14</v>
       </c>
       <c r="O192" s="7" t="n">
-        <v>0</v>
+        <v>0.85</v>
       </c>
       <c r="P192" s="7" t="n">
         <v>16.79</v>
       </c>
       <c r="Q192" s="7" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="R192" s="7" t="inlineStr">
         <is>
@@ -29409,19 +29409,19 @@
         <v>6894504330000</v>
       </c>
       <c r="M193" s="7" t="n">
-        <v>0.01</v>
+        <v>7.35</v>
       </c>
       <c r="N193" s="7" t="n">
-        <v>0.16</v>
+        <v>3.61</v>
       </c>
       <c r="O193" s="7" t="n">
-        <v>0</v>
+        <v>0.6</v>
       </c>
       <c r="P193" s="7" t="n">
         <v>8.77</v>
       </c>
       <c r="Q193" s="7" t="n">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="R193" s="7" t="inlineStr">
         <is>
@@ -29484,19 +29484,19 @@
         <v>7191120447000</v>
       </c>
       <c r="M194" s="7" t="n">
-        <v>0.01</v>
+        <v>13.73</v>
       </c>
       <c r="N194" s="7" t="n">
-        <v>-0.28</v>
+        <v>5.3</v>
       </c>
       <c r="O194" s="7" t="n">
-        <v>0</v>
+        <v>0.77</v>
       </c>
       <c r="P194" s="7" t="n">
         <v>5.71</v>
       </c>
       <c r="Q194" s="7" t="n">
-        <v>0</v>
+        <v>0.63</v>
       </c>
       <c r="R194" s="7" t="inlineStr">
         <is>
@@ -29559,17 +29559,17 @@
         <v>7555178683298.183</v>
       </c>
       <c r="M195" s="17" t="n">
-        <v>0.01</v>
+        <v>10.7</v>
       </c>
       <c r="N195" s="17" t="n"/>
       <c r="O195" s="17" t="n">
-        <v>0</v>
+        <v>0.84</v>
       </c>
       <c r="P195" s="17" t="n">
         <v>8.02</v>
       </c>
       <c r="Q195" s="17" t="n">
-        <v>0</v>
+        <v>0.66</v>
       </c>
       <c r="R195" s="17" t="inlineStr">
         <is>
@@ -29632,17 +29632,17 @@
         <v>7945504639144.696</v>
       </c>
       <c r="M196" s="17" t="n">
-        <v>0.01</v>
+        <v>9.98</v>
       </c>
       <c r="N196" s="17" t="n"/>
       <c r="O196" s="17" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="P196" s="17" t="n">
         <v>8.18</v>
       </c>
       <c r="Q196" s="17" t="n">
-        <v>0</v>
+        <v>0.64</v>
       </c>
       <c r="R196" s="17" t="inlineStr">
         <is>
@@ -36337,7 +36337,7 @@
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>2026-08-15T21:51:46+09:00</t>
+          <t>2026-08-15T21:58:11+09:00</t>
         </is>
       </c>
     </row>

</xml_diff>